<commit_message>
most finales changes 1 tag befor abgabe
- korrektur sven
- alle anhänge-
- teile neu geschrieben: prototyp zwei und finale lösung
</commit_message>
<xml_diff>
--- a/Morphologischer_Kasten/Morphologischer Kasten ausgefüllt.xlsx
+++ b/Morphologischer_Kasten/Morphologischer Kasten ausgefüllt.xlsx
@@ -425,13 +425,17 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -896,626 +900,626 @@
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
+      <c r="J3" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="3"/>
-      <c r="C5" s="4" t="s">
+      <c r="B5" s="4"/>
+      <c r="C5" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="4"/>
-      <c r="E5" s="5" t="s">
+      <c r="D5" s="5"/>
+      <c r="E5" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="F5" s="5"/>
-      <c r="G5" s="6" t="s">
+      <c r="F5" s="6"/>
+      <c r="G5" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="I5" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="J5" s="8"/>
+      <c r="J5" s="9"/>
     </row>
     <row r="6" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="10"/>
-      <c r="E6" s="11" t="s">
+      <c r="D6" s="11"/>
+      <c r="E6" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="F6" s="11"/>
-      <c r="G6" s="12" t="s">
+      <c r="F6" s="12"/>
+      <c r="G6" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="H6" s="13" t="s">
+      <c r="H6" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="I6" s="14" t="s">
+      <c r="I6" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="J6" s="15"/>
-      <c r="K6" s="16"/>
+      <c r="J6" s="16"/>
+      <c r="K6" s="17"/>
     </row>
     <row r="7" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="18"/>
-      <c r="E7" s="19" t="s">
+      <c r="D7" s="19"/>
+      <c r="E7" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="19"/>
-      <c r="G7" s="20" t="s">
+      <c r="F7" s="20"/>
+      <c r="G7" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="21" t="s">
+      <c r="H7" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="I7" s="14"/>
-      <c r="J7" s="22"/>
-      <c r="K7" s="23"/>
-      <c r="L7" s="23"/>
-      <c r="M7" s="23"/>
-      <c r="N7" s="23"/>
+      <c r="I7" s="15"/>
+      <c r="J7" s="23"/>
+      <c r="K7" s="24"/>
+      <c r="L7" s="24"/>
+      <c r="M7" s="24"/>
+      <c r="N7" s="24"/>
     </row>
     <row r="8" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="24" t="s">
+      <c r="C8" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="24"/>
-      <c r="E8" s="25" t="s">
+      <c r="D8" s="25"/>
+      <c r="E8" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="F8" s="25"/>
-      <c r="G8" s="26" t="s">
+      <c r="F8" s="26"/>
+      <c r="G8" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="H8" s="27" t="s">
+      <c r="H8" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="I8" s="28" t="s">
+      <c r="I8" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="J8" s="22"/>
-      <c r="K8" s="23"/>
-      <c r="L8" s="23"/>
-      <c r="M8" s="23"/>
-      <c r="N8" s="23"/>
+      <c r="J8" s="23"/>
+      <c r="K8" s="24"/>
+      <c r="L8" s="24"/>
+      <c r="M8" s="24"/>
+      <c r="N8" s="24"/>
     </row>
     <row r="9" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="29" t="s">
+      <c r="C9" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="29"/>
-      <c r="E9" s="19" t="s">
+      <c r="D9" s="30"/>
+      <c r="E9" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="F9" s="19"/>
-      <c r="G9" s="30" t="s">
+      <c r="F9" s="20"/>
+      <c r="G9" s="31" t="s">
         <v>26</v>
       </c>
-      <c r="H9" s="31"/>
-      <c r="I9" s="31"/>
-      <c r="J9" s="22"/>
-      <c r="K9" s="23"/>
-      <c r="L9" s="23"/>
-      <c r="M9" s="23"/>
-      <c r="N9" s="23"/>
+      <c r="H9" s="32"/>
+      <c r="I9" s="32"/>
+      <c r="J9" s="23"/>
+      <c r="K9" s="24"/>
+      <c r="L9" s="24"/>
+      <c r="M9" s="24"/>
+      <c r="N9" s="24"/>
     </row>
     <row r="10" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="32" t="s">
+      <c r="C10" s="33" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="32"/>
-      <c r="E10" s="33" t="s">
+      <c r="D10" s="33"/>
+      <c r="E10" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="F10" s="27" t="s">
+      <c r="F10" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="G10" s="14" t="s">
+      <c r="G10" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="H10" s="31"/>
-      <c r="I10" s="31"/>
-      <c r="J10" s="8"/>
-      <c r="K10" s="23"/>
-      <c r="L10" s="23"/>
-      <c r="N10" s="23"/>
+      <c r="H10" s="32"/>
+      <c r="I10" s="32"/>
+      <c r="J10" s="9"/>
+      <c r="K10" s="24"/>
+      <c r="L10" s="24"/>
+      <c r="N10" s="24"/>
     </row>
     <row r="11" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="32" t="s">
+      <c r="C11" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="D11" s="32"/>
-      <c r="E11" s="28" t="s">
+      <c r="D11" s="33"/>
+      <c r="E11" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="F11" s="28"/>
-      <c r="G11" s="30" t="s">
+      <c r="F11" s="29"/>
+      <c r="G11" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="H11" s="34" t="s">
+      <c r="H11" s="35" t="s">
         <v>36</v>
       </c>
-      <c r="I11" s="28" t="s">
+      <c r="I11" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="J11" s="8"/>
-      <c r="K11" s="23"/>
-      <c r="L11" s="23"/>
-      <c r="N11" s="23"/>
+      <c r="J11" s="9"/>
+      <c r="K11" s="24"/>
+      <c r="L11" s="24"/>
+      <c r="N11" s="24"/>
     </row>
     <row r="12" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="C12" s="35" t="s">
+      <c r="C12" s="36" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="35"/>
-      <c r="E12" s="33" t="s">
+      <c r="D12" s="36"/>
+      <c r="E12" s="34" t="s">
         <v>40</v>
       </c>
-      <c r="F12" s="33"/>
-      <c r="G12" s="36" t="s">
+      <c r="F12" s="34"/>
+      <c r="G12" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="H12" s="21"/>
-      <c r="I12" s="37"/>
-      <c r="J12" s="22"/>
-      <c r="K12" s="23"/>
-      <c r="L12" s="23"/>
-      <c r="N12" s="23"/>
+      <c r="H12" s="22"/>
+      <c r="I12" s="38"/>
+      <c r="J12" s="23"/>
+      <c r="K12" s="24"/>
+      <c r="L12" s="24"/>
+      <c r="N12" s="24"/>
     </row>
     <row r="13" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="C13" s="38" t="s">
+      <c r="C13" s="39" t="s">
         <v>43</v>
       </c>
-      <c r="D13" s="38"/>
-      <c r="E13" s="39" t="s">
+      <c r="D13" s="39"/>
+      <c r="E13" s="40" t="s">
         <v>44</v>
       </c>
-      <c r="F13" s="39"/>
-      <c r="G13" s="40" t="s">
+      <c r="F13" s="40"/>
+      <c r="G13" s="41" t="s">
         <v>45</v>
       </c>
-      <c r="H13" s="41" t="s">
+      <c r="H13" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="I13" s="42" t="s">
+      <c r="I13" s="43" t="s">
         <v>47</v>
       </c>
-      <c r="J13" s="22"/>
-      <c r="K13" s="23"/>
-      <c r="L13" s="23"/>
-      <c r="N13" s="23"/>
+      <c r="J13" s="23"/>
+      <c r="K13" s="24"/>
+      <c r="L13" s="24"/>
+      <c r="N13" s="24"/>
     </row>
     <row r="14" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="C14" s="43" t="s">
+      <c r="C14" s="44" t="s">
         <v>49</v>
       </c>
-      <c r="D14" s="43"/>
-      <c r="E14" s="28" t="s">
+      <c r="D14" s="44"/>
+      <c r="E14" s="29" t="s">
         <v>50</v>
       </c>
-      <c r="F14" s="28"/>
-      <c r="G14" s="19" t="s">
+      <c r="F14" s="29"/>
+      <c r="G14" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="H14" s="28" t="s">
+      <c r="H14" s="29" t="s">
         <v>52</v>
       </c>
-      <c r="I14" s="28"/>
-      <c r="J14" s="22"/>
-      <c r="K14" s="23"/>
-      <c r="L14" s="23"/>
-      <c r="N14" s="23"/>
+      <c r="I14" s="29"/>
+      <c r="J14" s="23"/>
+      <c r="K14" s="24"/>
+      <c r="L14" s="24"/>
+      <c r="N14" s="24"/>
     </row>
     <row r="15" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="17" t="s">
+      <c r="B15" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="C15" s="44" t="s">
+      <c r="C15" s="45" t="s">
         <v>54</v>
       </c>
-      <c r="D15" s="45"/>
-      <c r="E15" s="28" t="s">
+      <c r="D15" s="46"/>
+      <c r="E15" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="F15" s="28"/>
-      <c r="G15" s="27" t="s">
+      <c r="F15" s="29"/>
+      <c r="G15" s="28" t="s">
         <v>56</v>
       </c>
-      <c r="H15" s="28"/>
-      <c r="I15" s="31"/>
-      <c r="J15" s="22"/>
-      <c r="K15" s="23"/>
-      <c r="L15" s="23"/>
-      <c r="N15" s="23"/>
+      <c r="H15" s="29"/>
+      <c r="I15" s="32"/>
+      <c r="J15" s="23"/>
+      <c r="K15" s="24"/>
+      <c r="L15" s="24"/>
+      <c r="N15" s="24"/>
     </row>
     <row r="16" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="46"/>
-      <c r="C16" s="46"/>
-      <c r="D16" s="46"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="46"/>
-      <c r="H16" s="46"/>
-      <c r="I16" s="46"/>
-      <c r="J16" s="22"/>
-      <c r="K16" s="23"/>
-      <c r="L16" s="23"/>
-      <c r="N16" s="23"/>
+      <c r="B16" s="47"/>
+      <c r="C16" s="47"/>
+      <c r="D16" s="47"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="23"/>
+      <c r="G16" s="47"/>
+      <c r="H16" s="47"/>
+      <c r="I16" s="47"/>
+      <c r="J16" s="23"/>
+      <c r="K16" s="24"/>
+      <c r="L16" s="24"/>
+      <c r="N16" s="24"/>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="46"/>
-      <c r="C17" s="46"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22"/>
-      <c r="F17" s="22"/>
-      <c r="G17" s="22"/>
-      <c r="H17" s="22"/>
-      <c r="I17" s="22"/>
-      <c r="J17" s="22"/>
-      <c r="K17" s="23"/>
-      <c r="L17" s="23"/>
-      <c r="N17" s="23"/>
+      <c r="B17" s="47"/>
+      <c r="C17" s="47"/>
+      <c r="D17" s="23"/>
+      <c r="E17" s="23"/>
+      <c r="F17" s="23"/>
+      <c r="G17" s="23"/>
+      <c r="H17" s="23"/>
+      <c r="I17" s="23"/>
+      <c r="J17" s="23"/>
+      <c r="K17" s="24"/>
+      <c r="L17" s="24"/>
+      <c r="N17" s="24"/>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="46"/>
-      <c r="C18" s="46"/>
-      <c r="D18" s="22"/>
-      <c r="E18" s="22"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="22"/>
-      <c r="H18" s="22"/>
-      <c r="I18" s="22"/>
-      <c r="J18" s="22"/>
-      <c r="K18" s="23"/>
-      <c r="L18" s="23"/>
-      <c r="M18" s="23"/>
-      <c r="N18" s="23"/>
+      <c r="B18" s="47"/>
+      <c r="C18" s="47"/>
+      <c r="D18" s="23"/>
+      <c r="E18" s="23"/>
+      <c r="F18" s="23"/>
+      <c r="G18" s="23"/>
+      <c r="H18" s="23"/>
+      <c r="I18" s="23"/>
+      <c r="J18" s="23"/>
+      <c r="K18" s="24"/>
+      <c r="L18" s="24"/>
+      <c r="M18" s="24"/>
+      <c r="N18" s="24"/>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="46"/>
-      <c r="C19" s="46"/>
-      <c r="D19" s="15"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
-      <c r="G19" s="22"/>
-      <c r="H19" s="22"/>
-      <c r="I19" s="22"/>
-      <c r="J19" s="22"/>
-      <c r="K19" s="23"/>
-      <c r="L19" s="23"/>
-      <c r="M19" s="23"/>
-      <c r="N19" s="23"/>
+      <c r="B19" s="47"/>
+      <c r="C19" s="47"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="23"/>
+      <c r="F19" s="23"/>
+      <c r="G19" s="23"/>
+      <c r="H19" s="23"/>
+      <c r="I19" s="23"/>
+      <c r="J19" s="23"/>
+      <c r="K19" s="24"/>
+      <c r="L19" s="24"/>
+      <c r="M19" s="24"/>
+      <c r="N19" s="24"/>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="47"/>
-      <c r="C20" s="47"/>
-      <c r="D20" s="47"/>
-      <c r="E20" s="47"/>
-      <c r="F20" s="47"/>
-      <c r="G20" s="47"/>
-      <c r="H20" s="47"/>
-      <c r="I20" s="23"/>
-      <c r="J20" s="23"/>
-      <c r="K20" s="23"/>
-      <c r="L20" s="23"/>
-      <c r="M20" s="23"/>
-      <c r="N20" s="23"/>
+      <c r="B20" s="48"/>
+      <c r="C20" s="48"/>
+      <c r="D20" s="48"/>
+      <c r="E20" s="48"/>
+      <c r="F20" s="48"/>
+      <c r="G20" s="48"/>
+      <c r="H20" s="48"/>
+      <c r="I20" s="24"/>
+      <c r="J20" s="24"/>
+      <c r="K20" s="24"/>
+      <c r="L20" s="24"/>
+      <c r="M20" s="24"/>
+      <c r="N20" s="24"/>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="I21" s="23"/>
-      <c r="J21" s="23"/>
-      <c r="K21" s="23"/>
-      <c r="L21" s="23"/>
-      <c r="M21" s="23"/>
-      <c r="N21" s="23"/>
+      <c r="I21" s="24"/>
+      <c r="J21" s="24"/>
+      <c r="K21" s="24"/>
+      <c r="L21" s="24"/>
+      <c r="M21" s="24"/>
+      <c r="N21" s="24"/>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="48"/>
-      <c r="C22" s="48"/>
-      <c r="D22" s="48"/>
-      <c r="E22" s="48"/>
-      <c r="F22" s="48"/>
-      <c r="G22" s="48"/>
-      <c r="H22" s="48"/>
-      <c r="I22" s="23"/>
-      <c r="J22" s="23"/>
-      <c r="K22" s="23"/>
-      <c r="L22" s="23"/>
-      <c r="M22" s="23"/>
-      <c r="N22" s="23"/>
+      <c r="B22" s="49"/>
+      <c r="C22" s="49"/>
+      <c r="D22" s="49"/>
+      <c r="E22" s="49"/>
+      <c r="F22" s="49"/>
+      <c r="G22" s="49"/>
+      <c r="H22" s="49"/>
+      <c r="I22" s="24"/>
+      <c r="J22" s="24"/>
+      <c r="K22" s="24"/>
+      <c r="L22" s="24"/>
+      <c r="M22" s="24"/>
+      <c r="N22" s="24"/>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="48"/>
-      <c r="C23" s="48"/>
-      <c r="D23" s="48"/>
-      <c r="E23" s="48"/>
-      <c r="F23" s="48"/>
-      <c r="G23" s="48"/>
-      <c r="H23" s="48"/>
-      <c r="I23" s="23"/>
-      <c r="J23" s="23"/>
-      <c r="K23" s="23"/>
-      <c r="L23" s="23"/>
-      <c r="M23" s="23"/>
-      <c r="N23" s="23"/>
+      <c r="B23" s="49"/>
+      <c r="C23" s="49"/>
+      <c r="D23" s="49"/>
+      <c r="E23" s="49"/>
+      <c r="F23" s="49"/>
+      <c r="G23" s="49"/>
+      <c r="H23" s="49"/>
+      <c r="I23" s="24"/>
+      <c r="J23" s="24"/>
+      <c r="K23" s="24"/>
+      <c r="L23" s="24"/>
+      <c r="M23" s="24"/>
+      <c r="N23" s="24"/>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="48"/>
-      <c r="C24" s="48"/>
-      <c r="D24" s="48"/>
-      <c r="E24" s="48"/>
-      <c r="F24" s="48"/>
-      <c r="G24" s="48"/>
-      <c r="H24" s="48"/>
-      <c r="I24" s="23"/>
-      <c r="J24" s="23"/>
-      <c r="K24" s="23"/>
-      <c r="L24" s="23"/>
-      <c r="M24" s="23"/>
-      <c r="N24" s="23"/>
+      <c r="B24" s="49"/>
+      <c r="C24" s="49"/>
+      <c r="D24" s="49"/>
+      <c r="E24" s="49"/>
+      <c r="F24" s="49"/>
+      <c r="G24" s="49"/>
+      <c r="H24" s="49"/>
+      <c r="I24" s="24"/>
+      <c r="J24" s="24"/>
+      <c r="K24" s="24"/>
+      <c r="L24" s="24"/>
+      <c r="M24" s="24"/>
+      <c r="N24" s="24"/>
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="48"/>
-      <c r="C25" s="48"/>
-      <c r="D25" s="48"/>
-      <c r="E25" s="48"/>
-      <c r="F25" s="48"/>
-      <c r="G25" s="48"/>
-      <c r="H25" s="48"/>
-      <c r="I25" s="23"/>
-      <c r="J25" s="23"/>
-      <c r="K25" s="23"/>
-      <c r="L25" s="23"/>
-      <c r="M25" s="23"/>
-      <c r="N25" s="23"/>
+      <c r="B25" s="49"/>
+      <c r="C25" s="49"/>
+      <c r="D25" s="49"/>
+      <c r="E25" s="49"/>
+      <c r="F25" s="49"/>
+      <c r="G25" s="49"/>
+      <c r="H25" s="49"/>
+      <c r="I25" s="24"/>
+      <c r="J25" s="24"/>
+      <c r="K25" s="24"/>
+      <c r="L25" s="24"/>
+      <c r="M25" s="24"/>
+      <c r="N25" s="24"/>
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="48"/>
-      <c r="C26" s="48"/>
-      <c r="D26" s="48"/>
-      <c r="E26" s="48"/>
-      <c r="F26" s="48"/>
-      <c r="G26" s="48"/>
-      <c r="H26" s="48"/>
-      <c r="I26" s="23"/>
-      <c r="J26" s="23"/>
-      <c r="K26" s="23"/>
-      <c r="L26" s="23"/>
-      <c r="M26" s="23"/>
-      <c r="N26" s="23"/>
+      <c r="B26" s="49"/>
+      <c r="C26" s="49"/>
+      <c r="D26" s="49"/>
+      <c r="E26" s="49"/>
+      <c r="F26" s="49"/>
+      <c r="G26" s="49"/>
+      <c r="H26" s="49"/>
+      <c r="I26" s="24"/>
+      <c r="J26" s="24"/>
+      <c r="K26" s="24"/>
+      <c r="L26" s="24"/>
+      <c r="M26" s="24"/>
+      <c r="N26" s="24"/>
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="48"/>
-      <c r="C27" s="48"/>
-      <c r="D27" s="48"/>
-      <c r="E27" s="48"/>
-      <c r="F27" s="48"/>
-      <c r="G27" s="48"/>
-      <c r="H27" s="48"/>
-      <c r="I27" s="23"/>
-      <c r="J27" s="23"/>
-      <c r="K27" s="23"/>
-      <c r="L27" s="23"/>
-      <c r="M27" s="23"/>
-      <c r="N27" s="23"/>
+      <c r="B27" s="49"/>
+      <c r="C27" s="49"/>
+      <c r="D27" s="49"/>
+      <c r="E27" s="49"/>
+      <c r="F27" s="49"/>
+      <c r="G27" s="49"/>
+      <c r="H27" s="49"/>
+      <c r="I27" s="24"/>
+      <c r="J27" s="24"/>
+      <c r="K27" s="24"/>
+      <c r="L27" s="24"/>
+      <c r="M27" s="24"/>
+      <c r="N27" s="24"/>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="48"/>
-      <c r="C28" s="48"/>
-      <c r="D28" s="48"/>
-      <c r="E28" s="48"/>
-      <c r="F28" s="48"/>
-      <c r="G28" s="48"/>
-      <c r="H28" s="48"/>
-      <c r="I28" s="23"/>
-      <c r="J28" s="23"/>
-      <c r="K28" s="23"/>
-      <c r="L28" s="23"/>
-      <c r="M28" s="23"/>
-      <c r="N28" s="23"/>
+      <c r="B28" s="49"/>
+      <c r="C28" s="49"/>
+      <c r="D28" s="49"/>
+      <c r="E28" s="49"/>
+      <c r="F28" s="49"/>
+      <c r="G28" s="49"/>
+      <c r="H28" s="49"/>
+      <c r="I28" s="24"/>
+      <c r="J28" s="24"/>
+      <c r="K28" s="24"/>
+      <c r="L28" s="24"/>
+      <c r="M28" s="24"/>
+      <c r="N28" s="24"/>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="49"/>
-      <c r="C29" s="49"/>
-      <c r="D29" s="23"/>
-      <c r="E29" s="23"/>
-      <c r="F29" s="23"/>
-      <c r="G29" s="23"/>
-      <c r="H29" s="23"/>
-      <c r="I29" s="23"/>
-      <c r="J29" s="23"/>
-      <c r="K29" s="23"/>
-      <c r="L29" s="23"/>
-      <c r="M29" s="23"/>
-      <c r="N29" s="23"/>
+      <c r="B29" s="50"/>
+      <c r="C29" s="50"/>
+      <c r="D29" s="24"/>
+      <c r="E29" s="24"/>
+      <c r="F29" s="24"/>
+      <c r="G29" s="24"/>
+      <c r="H29" s="24"/>
+      <c r="I29" s="24"/>
+      <c r="J29" s="24"/>
+      <c r="K29" s="24"/>
+      <c r="L29" s="24"/>
+      <c r="M29" s="24"/>
+      <c r="N29" s="24"/>
     </row>
     <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="49"/>
-      <c r="C30" s="49"/>
-      <c r="D30" s="23"/>
-      <c r="E30" s="23"/>
-      <c r="F30" s="23"/>
-      <c r="G30" s="23"/>
-      <c r="H30" s="23"/>
-      <c r="I30" s="23"/>
-      <c r="J30" s="23"/>
-      <c r="K30" s="23"/>
-      <c r="L30" s="23"/>
-      <c r="M30" s="23"/>
-      <c r="N30" s="23"/>
+      <c r="B30" s="50"/>
+      <c r="C30" s="50"/>
+      <c r="D30" s="24"/>
+      <c r="E30" s="24"/>
+      <c r="F30" s="24"/>
+      <c r="G30" s="24"/>
+      <c r="H30" s="24"/>
+      <c r="I30" s="24"/>
+      <c r="J30" s="24"/>
+      <c r="K30" s="24"/>
+      <c r="L30" s="24"/>
+      <c r="M30" s="24"/>
+      <c r="N30" s="24"/>
     </row>
     <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="49"/>
-      <c r="C31" s="49"/>
-      <c r="D31" s="23"/>
-      <c r="E31" s="23"/>
-      <c r="F31" s="23"/>
-      <c r="G31" s="23"/>
-      <c r="H31" s="23"/>
-      <c r="I31" s="23"/>
-      <c r="J31" s="23"/>
-      <c r="K31" s="23"/>
-      <c r="L31" s="23"/>
-      <c r="M31" s="23"/>
-      <c r="N31" s="23"/>
+      <c r="B31" s="50"/>
+      <c r="C31" s="50"/>
+      <c r="D31" s="24"/>
+      <c r="E31" s="24"/>
+      <c r="F31" s="24"/>
+      <c r="G31" s="24"/>
+      <c r="H31" s="24"/>
+      <c r="I31" s="24"/>
+      <c r="J31" s="24"/>
+      <c r="K31" s="24"/>
+      <c r="L31" s="24"/>
+      <c r="M31" s="24"/>
+      <c r="N31" s="24"/>
     </row>
     <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="49"/>
-      <c r="C32" s="49"/>
-      <c r="D32" s="23"/>
-      <c r="E32" s="23"/>
-      <c r="F32" s="23"/>
-      <c r="G32" s="23"/>
-      <c r="H32" s="23"/>
-      <c r="I32" s="23"/>
-      <c r="J32" s="23"/>
-      <c r="K32" s="23"/>
-      <c r="L32" s="23"/>
-      <c r="M32" s="23"/>
-      <c r="N32" s="23"/>
+      <c r="B32" s="50"/>
+      <c r="C32" s="50"/>
+      <c r="D32" s="24"/>
+      <c r="E32" s="24"/>
+      <c r="F32" s="24"/>
+      <c r="G32" s="24"/>
+      <c r="H32" s="24"/>
+      <c r="I32" s="24"/>
+      <c r="J32" s="24"/>
+      <c r="K32" s="24"/>
+      <c r="L32" s="24"/>
+      <c r="M32" s="24"/>
+      <c r="N32" s="24"/>
     </row>
     <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B33" s="49"/>
-      <c r="C33" s="49"/>
-      <c r="D33" s="23"/>
-      <c r="E33" s="23"/>
-      <c r="F33" s="23"/>
-      <c r="G33" s="23"/>
-      <c r="H33" s="23"/>
-      <c r="I33" s="23"/>
-      <c r="J33" s="23"/>
-      <c r="K33" s="23"/>
-      <c r="L33" s="23"/>
-      <c r="M33" s="23"/>
-      <c r="N33" s="23"/>
+      <c r="B33" s="50"/>
+      <c r="C33" s="50"/>
+      <c r="D33" s="24"/>
+      <c r="E33" s="24"/>
+      <c r="F33" s="24"/>
+      <c r="G33" s="24"/>
+      <c r="H33" s="24"/>
+      <c r="I33" s="24"/>
+      <c r="J33" s="24"/>
+      <c r="K33" s="24"/>
+      <c r="L33" s="24"/>
+      <c r="M33" s="24"/>
+      <c r="N33" s="24"/>
     </row>
     <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B34" s="49"/>
-      <c r="C34" s="49"/>
-      <c r="D34" s="23"/>
-      <c r="E34" s="23"/>
-      <c r="F34" s="23"/>
-      <c r="G34" s="23"/>
-      <c r="H34" s="23"/>
-      <c r="I34" s="23"/>
-      <c r="J34" s="23"/>
-      <c r="K34" s="23"/>
-      <c r="L34" s="23"/>
-      <c r="M34" s="23"/>
-      <c r="N34" s="23"/>
+      <c r="B34" s="50"/>
+      <c r="C34" s="50"/>
+      <c r="D34" s="24"/>
+      <c r="E34" s="24"/>
+      <c r="F34" s="24"/>
+      <c r="G34" s="24"/>
+      <c r="H34" s="24"/>
+      <c r="I34" s="24"/>
+      <c r="J34" s="24"/>
+      <c r="K34" s="24"/>
+      <c r="L34" s="24"/>
+      <c r="M34" s="24"/>
+      <c r="N34" s="24"/>
     </row>
     <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B35" s="49"/>
-      <c r="C35" s="49"/>
-      <c r="D35" s="23"/>
-      <c r="E35" s="23"/>
-      <c r="F35" s="23"/>
-      <c r="G35" s="23"/>
-      <c r="H35" s="23"/>
-      <c r="I35" s="23"/>
-      <c r="J35" s="23"/>
-      <c r="K35" s="23"/>
-      <c r="L35" s="23"/>
-      <c r="M35" s="23"/>
-      <c r="N35" s="23"/>
+      <c r="B35" s="50"/>
+      <c r="C35" s="50"/>
+      <c r="D35" s="24"/>
+      <c r="E35" s="24"/>
+      <c r="F35" s="24"/>
+      <c r="G35" s="24"/>
+      <c r="H35" s="24"/>
+      <c r="I35" s="24"/>
+      <c r="J35" s="24"/>
+      <c r="K35" s="24"/>
+      <c r="L35" s="24"/>
+      <c r="M35" s="24"/>
+      <c r="N35" s="24"/>
     </row>
     <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B36" s="49"/>
-      <c r="C36" s="49"/>
-      <c r="D36" s="23"/>
-      <c r="E36" s="23"/>
-      <c r="F36" s="23"/>
-      <c r="G36" s="23"/>
-      <c r="H36" s="23"/>
-      <c r="I36" s="23"/>
-      <c r="J36" s="23"/>
-      <c r="K36" s="23"/>
-      <c r="L36" s="23"/>
-      <c r="M36" s="23"/>
-      <c r="N36" s="23"/>
+      <c r="B36" s="50"/>
+      <c r="C36" s="50"/>
+      <c r="D36" s="24"/>
+      <c r="E36" s="24"/>
+      <c r="F36" s="24"/>
+      <c r="G36" s="24"/>
+      <c r="H36" s="24"/>
+      <c r="I36" s="24"/>
+      <c r="J36" s="24"/>
+      <c r="K36" s="24"/>
+      <c r="L36" s="24"/>
+      <c r="M36" s="24"/>
+      <c r="N36" s="24"/>
     </row>
     <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B37" s="49"/>
-      <c r="C37" s="49"/>
-      <c r="D37" s="23"/>
-      <c r="E37" s="23"/>
-      <c r="F37" s="23"/>
-      <c r="G37" s="23"/>
-      <c r="H37" s="23"/>
-      <c r="I37" s="23"/>
-      <c r="J37" s="23"/>
-      <c r="K37" s="23"/>
-      <c r="L37" s="23"/>
-      <c r="M37" s="23"/>
-      <c r="N37" s="23"/>
+      <c r="B37" s="50"/>
+      <c r="C37" s="50"/>
+      <c r="D37" s="24"/>
+      <c r="E37" s="24"/>
+      <c r="F37" s="24"/>
+      <c r="G37" s="24"/>
+      <c r="H37" s="24"/>
+      <c r="I37" s="24"/>
+      <c r="J37" s="24"/>
+      <c r="K37" s="24"/>
+      <c r="L37" s="24"/>
+      <c r="M37" s="24"/>
+      <c r="N37" s="24"/>
     </row>
     <row r="38" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B38" s="49"/>
-      <c r="C38" s="49"/>
-      <c r="D38" s="23"/>
-      <c r="E38" s="23"/>
-      <c r="F38" s="23"/>
-      <c r="G38" s="23"/>
-      <c r="H38" s="23"/>
-      <c r="I38" s="23"/>
-      <c r="J38" s="23"/>
-      <c r="K38" s="23"/>
-      <c r="L38" s="23"/>
-      <c r="M38" s="23"/>
-      <c r="N38" s="23"/>
+      <c r="B38" s="50"/>
+      <c r="C38" s="50"/>
+      <c r="D38" s="24"/>
+      <c r="E38" s="24"/>
+      <c r="F38" s="24"/>
+      <c r="G38" s="24"/>
+      <c r="H38" s="24"/>
+      <c r="I38" s="24"/>
+      <c r="J38" s="24"/>
+      <c r="K38" s="24"/>
+      <c r="L38" s="24"/>
+      <c r="M38" s="24"/>
+      <c r="N38" s="24"/>
     </row>
     <row r="39" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B39" s="49"/>
-      <c r="C39" s="49"/>
-      <c r="D39" s="23"/>
-      <c r="E39" s="23"/>
-      <c r="F39" s="23"/>
-      <c r="G39" s="23"/>
-      <c r="H39" s="23"/>
-      <c r="I39" s="23"/>
-      <c r="J39" s="23"/>
-      <c r="K39" s="23"/>
-      <c r="L39" s="23"/>
-      <c r="M39" s="23"/>
-      <c r="N39" s="23"/>
+      <c r="B39" s="50"/>
+      <c r="C39" s="50"/>
+      <c r="D39" s="24"/>
+      <c r="E39" s="24"/>
+      <c r="F39" s="24"/>
+      <c r="G39" s="24"/>
+      <c r="H39" s="24"/>
+      <c r="I39" s="24"/>
+      <c r="J39" s="24"/>
+      <c r="K39" s="24"/>
+      <c r="L39" s="24"/>
+      <c r="M39" s="24"/>
+      <c r="N39" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="B3:J3"/>
+    <mergeCell ref="B3:I3"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="C6:D6"/>

</xml_diff>